<commit_message>
Deploy latest changes and restore local state
</commit_message>
<xml_diff>
--- a/public/assets/pompa mobile.xlsx
+++ b/public/assets/pompa mobile.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\program file\Project Kantor\System-sudin-jakarta-utara\public\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\program file\Project Kantor\Management Asset\public\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2E92FC98-045B-45BD-AEDC-0D3078B5F03D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B0D90E3D-3FF1-49B1-9E73-0DBEE538A951}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{4C65BAD7-D075-4324-9898-070247F9EF97}"/>
   </bookViews>

</xml_diff>